<commit_message>
Add QA report PRISM_Report_2026-05-31.xlsx
</commit_message>
<xml_diff>
--- a/reports/PRISM_Report_2026-05-31.xlsx
+++ b/reports/PRISM_Report_2026-05-31.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H37"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1007,9 +1007,373 @@
         <v/>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v/>
+      </c>
+      <c r="B24" t="str">
+        <v/>
+      </c>
+      <c r="C24" t="str">
+        <v/>
+      </c>
+      <c r="D24" t="str">
+        <v>FPS</v>
+      </c>
+      <c r="E24" t="str">
+        <v>29.91666666666667fps</v>
+      </c>
+      <c r="F24" t="str">
+        <v>29.91666666666667fps</v>
+      </c>
+      <c r="G24" t="str">
+        <v>29.91666666666667fps</v>
+      </c>
+      <c r="H24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Brightlight</v>
+      </c>
+      <c r="B25" t="str">
+        <v>1080p wide</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Front</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Wobble</v>
+      </c>
+      <c r="E25" t="str">
+        <v>No</v>
+      </c>
+      <c r="F25" t="str">
+        <v>No</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="H25" t="str">
+        <v>Video 1 has Brightness, Noise: Slight, Stability</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v/>
+      </c>
+      <c r="B26" t="str">
+        <v/>
+      </c>
+      <c r="C26" t="str">
+        <v/>
+      </c>
+      <c r="D26" t="str">
+        <v>Jitter</v>
+      </c>
+      <c r="E26" t="str">
+        <v>No</v>
+      </c>
+      <c r="F26" t="str">
+        <v>No</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="H26" t="str">
+        <v>Video 2 has Brightness, Noise, Stability</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v/>
+      </c>
+      <c r="B27" t="str">
+        <v/>
+      </c>
+      <c r="C27" t="str">
+        <v/>
+      </c>
+      <c r="D27" t="str">
+        <v>Brightness</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="G27" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="H27" t="str">
+        <v>Video 3 has Wobble, Jitter, Brightness, Noise, Stability</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v/>
+      </c>
+      <c r="B28" t="str">
+        <v/>
+      </c>
+      <c r="C28" t="str">
+        <v/>
+      </c>
+      <c r="D28" t="str">
+        <v>Noise</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Slight</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="H28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v/>
+      </c>
+      <c r="B29" t="str">
+        <v/>
+      </c>
+      <c r="C29" t="str">
+        <v/>
+      </c>
+      <c r="D29" t="str">
+        <v>Stability</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="G29" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="H29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v/>
+      </c>
+      <c r="B30" t="str">
+        <v/>
+      </c>
+      <c r="C30" t="str">
+        <v/>
+      </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
+      <c r="F30" t="str">
+        <v/>
+      </c>
+      <c r="G30" t="str">
+        <v/>
+      </c>
+      <c r="H30" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v/>
+      </c>
+      <c r="B31" t="str">
+        <v/>
+      </c>
+      <c r="C31" t="str">
+        <v/>
+      </c>
+      <c r="D31" t="str">
+        <v>FPS</v>
+      </c>
+      <c r="E31" t="str">
+        <v>29.91666666666667fps</v>
+      </c>
+      <c r="F31" t="str">
+        <v>29.91666666666667fps</v>
+      </c>
+      <c r="G31" t="str">
+        <v/>
+      </c>
+      <c r="H31" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Brightlight</v>
+      </c>
+      <c r="B32" t="str">
+        <v>1080p wide</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Front</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Wobble</v>
+      </c>
+      <c r="E32" t="str">
+        <v>No</v>
+      </c>
+      <c r="F32" t="str">
+        <v>No</v>
+      </c>
+      <c r="G32" t="str">
+        <v>—</v>
+      </c>
+      <c r="H32" t="str">
+        <v>Video 1 has Brightness, Noise: Slight, Stability</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v/>
+      </c>
+      <c r="B33" t="str">
+        <v/>
+      </c>
+      <c r="C33" t="str">
+        <v/>
+      </c>
+      <c r="D33" t="str">
+        <v>Jitter</v>
+      </c>
+      <c r="E33" t="str">
+        <v>No</v>
+      </c>
+      <c r="F33" t="str">
+        <v>No</v>
+      </c>
+      <c r="G33" t="str">
+        <v>—</v>
+      </c>
+      <c r="H33" t="str">
+        <v>Video 2 has Brightness, Noise, Stability</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v/>
+      </c>
+      <c r="B34" t="str">
+        <v/>
+      </c>
+      <c r="C34" t="str">
+        <v/>
+      </c>
+      <c r="D34" t="str">
+        <v>Brightness</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F34" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="G34" t="str">
+        <v>—</v>
+      </c>
+      <c r="H34" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v/>
+      </c>
+      <c r="B35" t="str">
+        <v/>
+      </c>
+      <c r="C35" t="str">
+        <v/>
+      </c>
+      <c r="D35" t="str">
+        <v>Noise</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Slight</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="G35" t="str">
+        <v>—</v>
+      </c>
+      <c r="H35" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v/>
+      </c>
+      <c r="B36" t="str">
+        <v/>
+      </c>
+      <c r="C36" t="str">
+        <v/>
+      </c>
+      <c r="D36" t="str">
+        <v>Stability</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="G36" t="str">
+        <v>—</v>
+      </c>
+      <c r="H36" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v/>
+      </c>
+      <c r="B37" t="str">
+        <v/>
+      </c>
+      <c r="C37" t="str">
+        <v/>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+      <c r="F37" t="str">
+        <v/>
+      </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
+      <c r="H37" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H37"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>